<commit_message>
just rolled back to the old methods
</commit_message>
<xml_diff>
--- a/annual-report-backend/data/processed/statement_jsons/Banking/NDB/2024/ndb_Banking_NDB_2024.xlsx
+++ b/annual-report-backend/data/processed/statement_jsons/Banking/NDB/2024/ndb_Banking_NDB_2024.xlsx
@@ -11,6 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="income_page_265" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="balance_page_267" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="cashflow_page_270" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="cashflow_page_271" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -456,7 +457,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-01-30T00:16:02.559164</t>
+          <t>2026-02-03T04:10:31.314028</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -7072,4 +7073,1633 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C95"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Key</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>For the year ended 31 December</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2024 (Bank)</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>For the year ended 31 December</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2023 (Bank)</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>For the year ended 31 December</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2024 (Group)</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>For the year ended 31 December</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2023 (Group)</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>LKR ’000 LKR ’000 LKR ’000 LKR ’000 Net (decrease)/increase in cash and cash equivalents</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2024 (Bank)</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>(21,667,326)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>LKR ’000 LKR ’000 LKR ’000 LKR ’000 Net (decrease)/increase in cash and cash equivalents</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>2023 (Bank)</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>22,938,775</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>LKR ’000 LKR ’000 LKR ’000 LKR ’000 Net (decrease)/increase in cash and cash equivalents</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>2024 (Group)</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>(21,502,738)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>LKR ’000 LKR ’000 LKR ’000 LKR ’000 Net (decrease)/increase in cash and cash equivalents</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2023 (Group)</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>22,540,792</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Cash and cash equivalents at the beginning of the year</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>2024 (Bank)</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>61,844,117</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Cash and cash equivalents at the beginning of the year</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>2023 (Bank)</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>38,958,510</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Cash and cash equivalents at the beginning of the year</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>2024 (Group)</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>62,324,278</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Cash and cash equivalents at the beginning of the year</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>2023 (Group)</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>39,836,654</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Cash and cash equivalents at the end of the year</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>2024 (Bank)</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>40,176,791</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Cash and cash equivalents at the end of the year</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>2023 (Bank)</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>61,897,285</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Cash and cash equivalents at the end of the year</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>2024 (Group)</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>40,821,540</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Cash and cash equivalents at the end of the year</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>2023 (Group)</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>62,377,446</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Reconciliation of cash and cash equivalents Cash and cash equivalents</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>2024 (Bank)</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>18,040,969</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Reconciliation of cash and cash equivalents Cash and cash equivalents</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>2023 (Bank)</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>28,104,415</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Reconciliation of cash and cash equivalents Cash and cash equivalents</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>2024 (Group)</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>18,685,718</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Reconciliation of cash and cash equivalents Cash and cash equivalents</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>2023 (Group)</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>28,584,576</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Placements with banks</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>2024 (Bank)</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>22,135,822</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Placements with banks</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>2023 (Bank)</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>33,792,870</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Placements with banks</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>2024 (Group)</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>22,135,822</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Placements with banks</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>2023 (Group)</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>33,792,870</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Cash and cash equivalents at the end of the year (Gross)</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>2024 (Bank)</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>40,176,791</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Cash and cash equivalents at the end of the year (Gross)</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>2023 (Bank)</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>61,897,285</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Cash and cash equivalents at the end of the year (Gross)</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>2024 (Group)</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>40,821,540</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Cash and cash equivalents at the end of the year (Gross)</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>2023 (Group)</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>62,377,446</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Less : Impairment allowance</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>2024 (Bank)</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>40,332</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Less : Impairment allowance</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>2023 (Bank)</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>53,168</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Less : Impairment allowance</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>2024 (Group)</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>40,332</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Less : Impairment allowance</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>2023 (Group)</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>53,168</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Cash and cash equivalents at the end of the year (Net)</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>2024 (Bank)</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>40,136,459</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Cash and cash equivalents at the end of the year (Net)</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>2023 (Bank)</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>61,844,117</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Cash and cash equivalents at the end of the year (Net)</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>2024 (Group)</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>40,781,208</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Cash and cash equivalents at the end of the year (Net)</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>2023 (Group)</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>62,324,278</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>LKR ’000 LKR ’000 LKR ’000 LKR ’000 Operating profit before tax on financial services</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>2024 (Bank)</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>24,342,991</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>LKR ’000 LKR ’000 LKR ’000 LKR ’000 Operating profit before tax on financial services</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>2023 (Bank)</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>10,095,757</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>LKR ’000 LKR ’000 LKR ’000 LKR ’000 Operating profit before tax on financial services</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>2024 (Group)</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>25,691,429</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>LKR ’000 LKR ’000 LKR ’000 LKR ’000 Operating profit before tax on financial services</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>2023 (Group)</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>10,904,079</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Gains on disposal of property, plant &amp; equipment</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>2024 (Bank)</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>(2,827)</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Gains on disposal of property, plant &amp; equipment</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>2023 (Bank)</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>(3,489)</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Gains on disposal of property, plant &amp; equipment</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>2024 (Group)</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>(2,827)</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Gains on disposal of property, plant &amp; equipment</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>2023 (Group)</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>(5,712)</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Accruals for interest/other income</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>2024 (Bank)</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>8,956,661</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Accruals for interest/other income</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>2023 (Bank)</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>(3,651,184)</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Accruals for interest/other income</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>2024 (Group)</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>9,026,743</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Accruals for interest/other income</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>2023 (Group)</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>(3,654,744)</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Accruals for interest expenses</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>2024 (Bank)</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>(6,522,277)</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Accruals for interest expenses</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>2023 (Bank)</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>(607,617)</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Accruals for interest expenses</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>2024 (Group)</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>(6,522,277)</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Accruals for interest expenses</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>2023 (Group)</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>(607,617)</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Accruals for general expenses</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>2024 (Bank)</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>(356,751)</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Accruals for general expenses</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>2023 (Bank)</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>(849,732)</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Accruals for general expenses</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>2024 (Group)</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>(583,128)</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Accruals for general expenses</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>2023 (Group)</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>(610,077)</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Unrealised revaluation gains/(losses) from investments</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>2024 (Bank)</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>(3,790,791)</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Unrealised revaluation gains/(losses) from investments</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>2023 (Bank)</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>(5,803,330)</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Unrealised revaluation gains/(losses) from investments</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>2024 (Group)</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>(4,268,055)</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Unrealised revaluation gains/(losses) from investments</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>2023 (Group)</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>(6,055,618)</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Contribution made to the pension fund</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>2024 (Bank)</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>(36,487)</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Contribution made to the pension fund</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>2023 (Bank)</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>(93,782)</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Contribution made to the pension fund</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>2024 (Group)</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>(36,487)</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Contribution made to the pension fund</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>2023 (Group)</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>(93,782)</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Depreciation of property, plant &amp; equipment</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>2024 (Bank)</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>401,609</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Depreciation of property, plant &amp; equipment</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>2023 (Bank)</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>393,336</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Depreciation of property, plant &amp; equipment</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>2024 (Group)</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>434,136</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Depreciation of property, plant &amp; equipment</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>2023 (Group)</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>420,837</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Amortisation of intangible assets</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>2024 (Bank)</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>313,001</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Amortisation of intangible assets</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>2023 (Bank)</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>271,056</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Amortisation of intangible assets</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>2024 (Group)</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>319,728</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Amortisation of intangible assets</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>2023 (Group)</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>275,353</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Depreciation of Right of use assets</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>2024 (Bank)</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>375,974</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Depreciation of Right of use assets</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>2023 (Bank)</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>320,118</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>Depreciation of Right of use assets</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>2024 (Group)</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>414,125</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>Depreciation of Right of use assets</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>2023 (Group)</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>358,269</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Impairment charges for financial assets and investments in subsidiaries</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>2024 (Bank)</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>(9,976,865)</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>Impairment charges for financial assets and investments in subsidiaries</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>2023 (Bank)</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>21,144,038</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>Impairment charges for financial assets and investments in subsidiaries</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>2024 (Group)</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>(10,054,600)</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>Impairment charges for financial assets and investments in subsidiaries</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>2023 (Group)</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>21,137,016</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>Loss on restructuring of Sri Lanka International Sovereign bonds (SLISBs)</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>2024 (Bank)</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>14,343,580</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>Loss on restructuring of Sri Lanka International Sovereign bonds (SLISBs)</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>2023 (Bank)</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>14,343,580</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>Scrip dividend received from investments</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>2024 (Bank)</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>(33,005)</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>Scrip dividend received from investments</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>2023 (Bank)</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>(41,932)</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>Scrip dividend received from investments</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>2024 (Group)</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>(40,129)</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>Scrip dividend received from investments</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>2023 (Group)</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>(42,075)</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>Share based expenses</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>2024 (Bank)</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>103,949</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>Share based expenses</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>2023 (Bank)</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>103,949</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>Fair value adjustments on investment property</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>2024 (Bank)</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>185,574</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>Fair value adjustments on investment property</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>2023 (Bank)</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>(211,552)</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>Operating profit before changes in operating assets and liabilities</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>2024 (Bank)</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>28,118,762</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>Operating profit before changes in operating assets and liabilities</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>2023 (Bank)</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>21,173,239</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>Operating profit before changes in operating assets and liabilities</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>2024 (Group)</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>29,011,761</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>Operating profit before changes in operating assets and liabilities</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>2023 (Group)</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>21,814,377</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>